<commit_message>
feat: add paddleOCR e DocTR
</commit_message>
<xml_diff>
--- a/docs/planejamento_modelos.xlsx
+++ b/docs/planejamento_modelos.xlsx
@@ -601,9 +601,9 @@
           <t>src/ocr/classical/paddleocr_ocr.py</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -628,9 +628,9 @@
           <t>src/ocr/classical/doctr_ocr.py</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: wire MODEL_REGISTRY and update deps for all 13 OCR models
</commit_message>
<xml_diff>
--- a/docs/planejamento_modelos.xlsx
+++ b/docs/planejamento_modelos.xlsx
@@ -655,9 +655,9 @@
           <t>src/ocr/transformer/trocr_base.py</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -682,9 +682,9 @@
           <t>src/ocr/transformer/trocr_large.py</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -709,9 +709,9 @@
           <t>src/ocr/vlm/gemma_ocr.py</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -736,9 +736,9 @@
           <t>src/ocr/vlm/deepseek_ocr.py</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -763,9 +763,9 @@
           <t>src/ocr/vlm/qwen_ocr.py</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -790,9 +790,9 @@
           <t>src/ocr/vlm/llamaparse_ocr.py</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -817,9 +817,9 @@
           <t>src/ocr/vlm/mistral_ocr.py</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -844,9 +844,9 @@
           <t>src/ocr/vlm/gemini_ocr.py</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -871,9 +871,9 @@
           <t>src/ocr/__init__.py (+ subpacotes)</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -925,9 +925,9 @@
           <t>requirements.txt: adicionar deps novas (transformers, torch, craft-text-detector, ollama, llama-parse, mistralai, google-generativeai, jiwer, python-dotenv)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -942,9 +942,9 @@
           <t>.env.example (LLAMA_CLOUD_API_KEY, MISTRAL_API_KEY, GEMINI_API_KEY)</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: implement PDF to PNG conversion
</commit_message>
<xml_diff>
--- a/docs/planejamento_modelos.xlsx
+++ b/docs/planejamento_modelos.xlsx
@@ -1019,9 +1019,9 @@
           <t>converter.py: implementar conversão PDF -&gt; PNG (pdf2image)</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: track time/memory/tokens per page and export full Excel report
</commit_message>
<xml_diff>
--- a/docs/planejamento_modelos.xlsx
+++ b/docs/planejamento_modelos.xlsx
@@ -982,7 +982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -1063,9 +1063,9 @@
           <t>run_benchmark.py: implementar loop de execução + chamada a metrics.py</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1085,9 +1085,9 @@
           <t>metrics.py: implementar iteração sobre páginas em evaluate_model</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1186,6 +1186,50 @@
       <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Necessário para rodar os modelos via API</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>manifest.csv: obra/página/dificuldade (Tabela 4.4 do TCC)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>benchmark/ground_truth/manifest.csv, 20 páginas — pronto para casar com os .txt de regra ouro</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>run_benchmark.py: métricas de custo (tempo, memória RAM/GPU, tokens) + planilha Excel</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>benchmark_resultados.xlsx com abas Resultados e Resumo por Modelo; testado com modelo falso</t>
         </is>
       </c>
     </row>

</xml_diff>